<commit_message>
optimize file_path,add coroutine rpc api, cmake modify pb
</commit_message>
<xml_diff>
--- a/config/excel/ServerList.xlsx
+++ b/config/excel/ServerList.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\proj\server_demo\config\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Proj\demo1\config\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B3DFBF-A2FE-4C83-912C-AEA08CE33811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16200" yWindow="408" windowWidth="20448" windowHeight="20592"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ServerList" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>Id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -90,58 +91,62 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>[int32]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ServerIp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>服务器地址</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>服务对外地址</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>string</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>string</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PublicIp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>127.0.0.1 9997</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>int32</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>网络线程数量</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NetThreadsNum</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dbSercer</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>127.0.0.1 9999</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[int32]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ServerIp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>服务器地址</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>服务对外地址</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>string</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>string</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PublicIp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>127.0.0.1 9997</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>int32</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>网络线程数量</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NetThreadsNum</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -459,20 +464,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:H6"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A2:H7"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.21875" customWidth="1"/>
+    <col min="4" max="4" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.25" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>10</v>
       </c>
@@ -483,19 +488,19 @@
         <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G2" t="s">
         <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -509,19 +514,19 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -535,19 +540,19 @@
         <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G4" t="s">
         <v>6</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>10001</v>
       </c>
@@ -561,19 +566,19 @@
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G5">
         <v>2</v>
       </c>
       <c r="H5">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>20001</v>
       </c>
@@ -587,13 +592,36 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G6">
         <v>1</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>30001</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>